<commit_message>
Import all 10 Novixa news articles from Excel
</commit_message>
<xml_diff>
--- a/novixa-site/import/tin-tuc.xlsx
+++ b/novixa-site/import/tin-tuc.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PharmaCore\novixa-site\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PharmaCore\novixa-site\import\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>title</t>
   </si>
@@ -41,17 +41,40 @@
     <t>content</t>
   </si>
   <si>
-    <t>Mô tả ngắn 1–2 câu (SEO, danh sách tin)</t>
-  </si>
-  <si>
     <t>Quản lý nhà thuốc thông minh — từ quầy bán đến tồn kho lô</t>
   </si>
   <si>
     <t>22-6-2026</t>
   </si>
   <si>
-    <t xml:space="preserve"># Quản lý nhà thuốc thông minh — từ quầy bán đến tồn kho lô
-Nhiều nhà thuốc hiện nay vẫn đang vận hành theo cách quen thuộc: ghi nhớ bằng kinh nghiệm, quản lý tồn kho bằng Excel, kiểm tra hạn dùng bằng mắt và xử lý công nợ thủ công. Khi quy mô còn nhỏ, cách làm này có thể đáp ứng được. Nhưng khi lượng hàng hóa tăng lên hàng nghìn sản phẩm, hàng chục nhà cung cấp và hàng trăm khách hàng mỗi ngày, những rủi ro bắt đầu xuất hiện.
+    <t>7 Sai Lầm Khiến Nhà Thuốc Thất Thoát Lợi Nhuận Mỗi Tháng</t>
+  </si>
+  <si>
+    <t>23-6-2026</t>
+  </si>
+  <si>
+    <t>24-26-2026</t>
+  </si>
+  <si>
+    <t>25-6-2026</t>
+  </si>
+  <si>
+    <t>26-6-2026</t>
+  </si>
+  <si>
+    <t>27-6-2026</t>
+  </si>
+  <si>
+    <t>28-6-2026</t>
+  </si>
+  <si>
+    <t>29-6-2026</t>
+  </si>
+  <si>
+    <t>30-6-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nhiều nhà thuốc hiện nay vẫn đang vận hành theo cách quen thuộc: ghi nhớ bằng kinh nghiệm, quản lý tồn kho bằng Excel, kiểm tra hạn dùng bằng mắt và xử lý công nợ thủ công. Khi quy mô còn nhỏ, cách làm này có thể đáp ứng được. Nhưng khi lượng hàng hóa tăng lên hàng nghìn sản phẩm, hàng chục nhà cung cấp và hàng trăm khách hàng mỗi ngày, những rủi ro bắt đầu xuất hiện.
 Một sản phẩm hết hạn không được phát hiện kịp thời.
 Một lô thuốc bị thu hồi nhưng không xác định được đã bán cho ai.
 Một mặt hàng tồn kho quá lâu làm chôn vốn.
@@ -123,14 +146,7 @@
 </t>
   </si>
   <si>
-    <t>7 Sai Lầm Khiến Nhà Thuốc Thất Thoát Lợi Nhuận Mỗi Tháng</t>
-  </si>
-  <si>
-    <t>23-6-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># 7 Sai Lầm Khiến Nhà Thuốc Thất Thoát Lợi Nhuận Mỗi Tháng
-Nhiều chủ nhà thuốc cho rằng lợi nhuận giảm là do cạnh tranh hoặc giá nhập tăng. Tuy nhiên, thực tế cho thấy phần lớn thất thoát đến từ các sai sót trong quản lý hàng ngày.
+    <t xml:space="preserve">Nhiều chủ nhà thuốc cho rằng lợi nhuận giảm là do cạnh tranh hoặc giá nhập tăng. Tuy nhiên, thực tế cho thấy phần lớn thất thoát đến từ các sai sót trong quản lý hàng ngày.
 ## 1. Không quản lý tồn kho theo lô
 Hai hộp thuốc cùng tên nhưng khác số lô và hạn sử dụng có giá trị hoàn toàn khác nhau. Nếu chỉ theo dõi số lượng tổng, nhà thuốc rất dễ bỏ sót hàng sắp hết hạn.
 ## 2. Không kiểm tra hàng cận date thường xuyên
@@ -150,40 +166,7 @@
 </t>
   </si>
   <si>
-    <t>Vì Sao Excel Không Còn Phù Hợp Để Quản Lý Nhà Thuốc?</t>
-  </si>
-  <si>
-    <t>24-26-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># Vì Sao Excel Không Còn Phù Hợp Để Quản Lý Nhà Thuốc?
-Excel từng là công cụ quen thuộc của rất nhiều nhà thuốc. Tuy nhiên khi quy mô kinh doanh tăng lên, những hạn chế của Excel bắt đầu bộc lộ rõ ràng.
-## Khó quản lý số lượng sản phẩm lớn
-Một nhà thuốc trung bình có thể kinh doanh từ 2.000 đến 5.000 sản phẩm. Việc cập nhật thủ công dễ dẫn đến sai sót và mất thời gian.
-## Không quản lý được lô và hạn dùng hiệu quả
-Excel có thể lưu dữ liệu nhưng không thể tự động cảnh báo hàng cận date hoặc đề xuất xuất trước các lô gần hết hạn.
-## Dễ xảy ra sai sót khi nhiều người cùng làm việc
-Khi nhiều nhân viên cùng chỉnh sửa một file, nguy cơ ghi đè dữ liệu hoặc nhập sai thông tin là rất cao.
-## Không hỗ trợ bán hàng thời gian thực
-Khi bán một sản phẩm, tồn kho cần được cập nhật ngay lập tức. Excel không được thiết kế cho mục đích này.
-## Không có cảnh báo thông minh
-Excel không tự động nhắc nhập hàng, cảnh báo tồn kho thấp hay phân tích doanh thu.
-## Khó mở rộng khi có nhiều chi nhánh
-Việc tổng hợp dữ liệu từ nhiều file Excel khác nhau rất phức tạp và dễ sai lệch.
-## Không hỗ trợ CRM
-Excel không thể quản lý lịch sử mua hàng, điểm tích lũy hay chương trình chăm sóc khách hàng một cách hiệu quả.
-## Kết luận
-Excel vẫn phù hợp cho những cửa hàng rất nhỏ. Tuy nhiên, để phát triển bền vững và cạnh tranh trong thời đại số, nhà thuốc cần một hệ thống quản lý chuyên nghiệp có khả năng quản lý tồn kho, bán hàng, khách hàng và dữ liệu tập trung.
-</t>
-  </si>
-  <si>
-    <t>Quản Lý Tồn Kho Thuốc Hiệu Quả Cho Nhà Thuốc Hiện Đại</t>
-  </si>
-  <si>
-    <t>25-6-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># Quản Lý Tồn Kho Thuốc Hiệu Quả Cho Nhà Thuốc Hiện Đại
+    <t xml:space="preserve">
 Tồn kho là tài sản lớn nhất của hầu hết các nhà thuốc. Quản lý tồn kho tốt giúp tăng lợi nhuận, giảm thất thoát và cải thiện dòng tiền.
 ## Tại sao tồn kho quan trọng?
 Mỗi sản phẩm nằm trên kệ đều là vốn của doanh nghiệp. Nếu hàng hóa lưu kho quá lâu, vốn sẽ bị chôn và hiệu quả kinh doanh giảm xuống.
@@ -209,14 +192,26 @@
 </t>
   </si>
   <si>
-    <t>Làm Sao Kiểm Soát Hàng Cận Date Và Hết Hạn Trong Nhà Thuốc?</t>
-  </si>
-  <si>
-    <t>26-6-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># Làm Sao Kiểm Soát Hàng Cận Date Và Hết Hạn Trong Nhà Thuốc?
-Một trong những nguyên nhân gây thất thoát lớn nhất tại nhà thuốc là hàng hóa hết hạn sử dụng. Không chỉ gây thiệt hại về tài chính, việc bán nhầm sản phẩm hết hạn còn ảnh hưởng nghiêm trọng đến uy tín và có thể dẫn đến các vấn đề pháp lý.
+    <t xml:space="preserve">Excel từng là công cụ quen thuộc của rất nhiều nhà thuốc. Tuy nhiên khi quy mô kinh doanh tăng lên, những hạn chế của Excel bắt đầu bộc lộ rõ ràng.
+## Khó quản lý số lượng sản phẩm lớn
+Một nhà thuốc trung bình có thể kinh doanh từ 2.000 đến 5.000 sản phẩm. Việc cập nhật thủ công dễ dẫn đến sai sót và mất thời gian.
+## Không quản lý được lô và hạn dùng hiệu quả
+Excel có thể lưu dữ liệu nhưng không thể tự động cảnh báo hàng cận date hoặc đề xuất xuất trước các lô gần hết hạn.
+## Dễ xảy ra sai sót khi nhiều người cùng làm việc
+Khi nhiều nhân viên cùng chỉnh sửa một file, nguy cơ ghi đè dữ liệu hoặc nhập sai thông tin là rất cao.
+Khi bán một sản phẩm, tồn kho cần được cập nhật ngay lập tức. Excel không được thiết kế cho mục đích này.
+## Không có cảnh báo thông minh
+Excel không tự động nhắc nhập hàng, cảnh báo tồn kho thấp hay phân tích doanh thu.
+## Khó mở rộng khi có nhiều chi nhánh
+Việc tổng hợp dữ liệu từ nhiều file Excel khác nhau rất phức tạp và dễ sai lệch.
+## Không hỗ trợ CRM
+Excel không thể quản lý lịch sử mua hàng, điểm tích lũy hay chương trình chăm sóc khách hàng một cách hiệu quả.
+## Kết luận
+Excel vẫn phù hợp cho những cửa hàng rất nhỏ. Tuy nhiên, để phát triển bền vững và cạnh tranh trong thời đại số, nhà thuốc cần một hệ thống quản lý chuyên nghiệp có khả năng quản lý tồn kho, bán hàng, khách hàng và dữ liệu tập trung.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Một trong những nguyên nhân gây thất thoát lớn nhất tại nhà thuốc là hàng hóa hết hạn sử dụng. Không chỉ gây thiệt hại về tài chính, việc bán nhầm sản phẩm hết hạn còn ảnh hưởng nghiêm trọng đến uy tín và có thể dẫn đến các vấn đề pháp lý.
 ## Vì sao hàng cận date là vấn đề lớn?
 Nhiều chủ nhà thuốc chỉ phát hiện sản phẩm sắp hết hạn khi kiểm kê định kỳ. Khi đó thời gian xử lý thường không còn nhiều, dẫn đến việc giảm giá sâu hoặc tiêu hủy hàng hóa.
 Những nguyên nhân phổ biến gồm:
@@ -251,13 +246,7 @@
 </t>
   </si>
   <si>
-    <t>FEFO Là Gì Và Tại Sao Nhà Thuốc Nên Áp Dụng?</t>
-  </si>
-  <si>
-    <t>27-6-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># FEFO Là Gì Và Tại Sao Nhà Thuốc Nên Áp Dụng?
+    <t xml:space="preserve">
 Trong ngành dược, việc xuất bán đúng lô hàng quan trọng không kém việc nhập hàng đúng giá. FEFO là một trong những nguyên tắc giúp nhà thuốc giảm thất thoát và đảm bảo chất lượng sản phẩm.
 ## FEFO là gì?
 FEFO là viết tắt của:
@@ -305,13 +294,7 @@
 </t>
   </si>
   <si>
-    <t>Quản Lý Nhiều Chi Nhánh Nhà Thuốc Như Thế Nào?</t>
-  </si>
-  <si>
-    <t>28-6-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># Quản Lý Nhiều Chi Nhánh Nhà Thuốc Như Thế Nào?
+    <t xml:space="preserve">
 Khi mở thêm chi nhánh thứ hai, thứ ba, nhiều chủ nhà thuốc nhận ra rằng việc quản lý không còn đơn giản như trước.
 Thách thức không nằm ở bán hàng mà nằm ở dữ liệu.
 ## Những khó khăn phổ biến
@@ -362,13 +345,7 @@
 </t>
   </si>
   <si>
-    <t>Cách Giảm Tồn Kho Chết Trong Nhà Thuốc</t>
-  </si>
-  <si>
-    <t>29-6-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># Cách Giảm Tồn Kho Chết Trong Nhà Thuốc
+    <t xml:space="preserve">
 Tồn kho là tài sản của nhà thuốc. Tuy nhiên, không phải hàng tồn nào cũng mang lại giá trị. Một phần hàng hóa có thể nằm trên kệ nhiều tháng, thậm chí nhiều năm mà không phát sinh giao dịch. Đây chính là tồn kho chết.
 Tồn kho chết không chỉ chiếm diện tích lưu trữ mà còn làm giảm dòng tiền, tăng nguy cơ hết hạn và ảnh hưởng trực tiếp đến lợi nhuận.
 ## Tồn kho chết là gì?
@@ -418,14 +395,7 @@
 </t>
   </si>
   <si>
-    <t>Chuyển Đổi Số Nhà Thuốc Bắt Đầu Từ Đâu?</t>
-  </si>
-  <si>
-    <t>30-6-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># Chuyển Đổi Số Nhà Thuốc Bắt Đầu Từ Đâu?
-Chuyển đổi số đang trở thành xu hướng tất yếu trong ngành dược. Tuy nhiên, nhiều chủ nhà thuốc vẫn nghĩ rằng chuyển đổi số là một dự án phức tạp và tốn kém.
+    <t xml:space="preserve">Chuyển đổi số đang trở thành xu hướng tất yếu trong ngành dược. Tuy nhiên, nhiều chủ nhà thuốc vẫn nghĩ rằng chuyển đổi số là một dự án phức tạp và tốn kém.
 Thực tế, chuyển đổi số bắt đầu từ những bước rất cơ bản.
 ## Chuyển đổi số không phải là mua phần mềm
 Nhiều người nhầm tưởng:
@@ -478,10 +448,7 @@
 </t>
   </si>
   <si>
-    <t>Các Chỉ Số KPI Quan Trọng Của Nhà Thuốc</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># Các Chỉ Số KPI Quan Trọng Của Nhà Thuốc
+    <t xml:space="preserve">
 Một trong những sai lầm phổ biến của chủ nhà thuốc là chỉ theo dõi doanh thu. Thực tế, doanh thu cao chưa chắc đồng nghĩa với hiệu quả kinh doanh tốt.
 Để quản lý nhà thuốc chuyên nghiệp, cần theo dõi các KPI quan trọng.
 ## 1. Doanh thu
@@ -906,118 +873,88 @@
     </row>
     <row r="2" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C6" s="1" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="1" t="s">
+    </row>
+    <row r="8" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="1" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="1" t="s">
+    <row r="10" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="11" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="C11" s="3">
         <v>46029</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>